<commit_message>
Documente les reponses 13 et 14, la lecture des CSV et le stockage plein
Q13 : tout l'historique, tout type de fichier (priorite des 17 fichiers a
preciser). Q14 : a voir avec le delegue a la protection des donnees, pas
encore sollicite - decision a obtenir avant le choix de l'hebergeur.
Plan de mise en production : volume mesure d'un historique complet (proche de
la limite du navigateur), decisions a jour. Kit regenere : regle des formats
acceptes. ETAT, CLAUDE.md (composant import-fichier), BUGS-CONNUS, checklist
a 125 points, point de reprise.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KIT-REPRISE/00-mode-d-emploi.xlsx
+++ b/KIT-REPRISE/00-mode-d-emploi.xlsx
@@ -843,7 +843,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -862,27 +862,32 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Respectez l'ordre des fichiers : certains se rattachent à des données chargées avant (accidents, trames, catalogue d'EPI).</v>
+        <v>Formats acceptés : Excel (.xlsx, .xls), LibreOffice (.ods) et CSV (séparateur point-virgule ou virgule, quel que soit l'encodage). Un document Word, PDF ou papier, ou l'export d'un autre logiciel sous un autre format, se recopie d'abord dans le modèle.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Après chaque import, l'application affiche combien de lignes ont été ajoutées, mises à jour ou ignorées : notez les lignes ignorées et corrigez-les.</v>
+        <v>Respectez l'ordre des fichiers : certains se rattachent à des données chargées avant (accidents, trames, catalogue d'EPI).</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Un fichier réimporté met à jour les lignes qu'il reconnaît ; une colonne absente du fichier ne modifie pas ce qui est déjà enregistré (Gestion RH, Dossiers AT/MP).</v>
+        <v>Après chaque import, l'application affiche combien de lignes ont été ajoutées, mises à jour ou ignorées : notez les lignes ignorées et corrigez-les.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>Un fichier réimporté met à jour les lignes qu'il reconnaît ; une colonne absente du fichier ne modifie pas ce qui est déjà enregistré (Gestion RH, Dossiers AT/MP).</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
         <v>Les données restent aujourd'hui dans le navigateur qui les importe : faites la reprise sur le poste qui servira, et gardez vos fichiers.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Kit de reprise complet : referentiels importables, arbre causal repris
KIT-REPRISE : nouveau modele 00-referentiels.xlsx, a charger en premier (la
saisie a la main des referentiels n'est plus une etape prealable) ; le modele
des analyses d'accident porte les feuilles Faits, Pourquoi et Ishikawa. 18
modeles, tous importables, consignes mesurees.
Generateur : session par module (Administration), comptage relatif aux
valeurs par defaut, referentiels non repris comme prerequis d'eux-memes.

Documentation : ETAT (Administration, Analyse d'accident), BUGS-CONNUS
(actions dupliquees au reimport), checklist a 127 points, plan de mise en
production, point de reprise.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KIT-REPRISE/00-mode-d-emploi.xlsx
+++ b/KIT-REPRISE/00-mode-d-emploi.xlsx
@@ -434,30 +434,30 @@
         <v>(saisie à l'écran)</v>
       </c>
       <c r="C2" t="str">
-        <v>Référentiels (services, sites, familles de risque…)</v>
+        <v>Comptes utilisateurs</v>
       </c>
       <c r="D2" t="str">
-        <v>Administration → Référentiels</v>
+        <v>Administration → Utilisateurs</v>
       </c>
       <c r="E2" t="str">
-        <v>À faire AVANT tout import : les colonnes « Service » des fichiers doivent reprendre exactement ces libellés.</v>
+        <v>Créés un par un (ils relèveront de la future authentification).</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Avant</v>
+        <v>00</v>
       </c>
       <c r="B3" t="str">
-        <v>(saisie à l'écran)</v>
+        <v>00-referentiels.xlsx</v>
       </c>
       <c r="C3" t="str">
-        <v>Comptes utilisateurs</v>
+        <v>Référentiels (services, familles de risque, listes)</v>
       </c>
       <c r="D3" t="str">
-        <v>Administration → Utilisateurs</v>
+        <v>Administration → Référentiels → Importer .xlsx</v>
       </c>
       <c r="E3" t="str">
-        <v>Créés un par un (ils relèveront de la future authentification).</v>
+        <v>À charger en tout premier : les colonnes « Service » des autres fichiers doivent reprendre exactement ces libellés. L'import ajoute les valeurs manquantes et n'en retire jamais ; la colonne « Définition » ne sert qu'aux familles de risque.</v>
       </c>
     </row>
     <row r="4">
@@ -474,7 +474,7 @@
         <v>Gestion RH → onglet Agents → Importer .xlsx</v>
       </c>
       <c r="E4" t="str">
-        <v>À charger en premier : les autres modules peuvent ensuite proposer ces agents dans leurs formulaires. Le responsable se désigne par son « Nom Prénom » ; il peut figurer plus bas dans le fichier.</v>
+        <v>À charger juste après les référentiels : les autres modules peuvent ensuite proposer ces agents dans leurs formulaires. Le responsable se désigne par son « Nom Prénom » ; il peut figurer plus bas dans le fichier.</v>
       </c>
     </row>
     <row r="5">
@@ -542,7 +542,7 @@
         <v>Analyse d'accident → Importer .xlsx</v>
       </c>
       <c r="E8" t="str">
-        <v>La méthode, la conclusion et les actions correctives se reprennent ; l'arbre des causes lui-même (faits, « pourquoi », diagramme d'Ishikawa) se ressaisit à l'écran — la page le signale à l'import.</v>
+        <v>La méthode, la conclusion, les actions correctives et l'arbre causal (feuilles « Faits », « Pourquoi », « Ishikawa ») se reprennent. Dans « Faits », la colonne « Découle du fait n° » désigne un autre fait de la même analyse par son numéro.</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
J1 : objectifs santé-sécurité (ISO 45001 § 6.2), repris par la revue de direction
Page objectifs.html (Pilotage, droit « objectifs ») : cible chiffrée sur un indicateur
calculé par assets/indicateurs.js (ou mesure manuelle), écart et état du jour sans prorata,
moyens, actions au Plan d'actions (origine « Objectif »), résultat figé à la clôture.
Catalogue et lecture partagés : assets/objectifs-ref.js. indicateurs.js rend aussi le TG
estimé (Reporting inchangé, 35/35). Revue de direction : objectifs de la période dans
« Politique et objectifs ». Question 24 au préventeur. Checklist QA : 207 points.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KIT-REPRISE/00-mode-d-emploi.xlsx
+++ b/KIT-REPRISE/00-mode-d-emploi.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <cols>
     <col min="1" max="1" width="7.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -789,13 +789,13 @@
         <v>(saisie à l'écran)</v>
       </c>
       <c r="C23" t="str">
-        <v>Revues de direction</v>
+        <v>Objectifs santé-sécurité</v>
       </c>
       <c r="D23" t="str">
-        <v>Revue de direction</v>
+        <v>Objectifs santé-sécurité</v>
       </c>
       <c r="E23" t="str">
-        <v>Pas d'import : chaque revue se prépare à l'écran à partir des données reprises.</v>
+        <v>Pas d'import : chaque objectif se fixe à l'écran, sur un indicateur que l'application calcule.</v>
       </c>
     </row>
     <row r="24">
@@ -806,13 +806,13 @@
         <v>(saisie à l'écran)</v>
       </c>
       <c r="C24" t="str">
-        <v>Signalements</v>
+        <v>Revues de direction</v>
       </c>
       <c r="D24" t="str">
-        <v>Signalements</v>
+        <v>Revue de direction</v>
       </c>
       <c r="E24" t="str">
-        <v>Pas d'import : chaque presque-accident se signale à l'écran ; un historique se reprend au Registre AT/MP (type « Presque accident »).</v>
+        <v>Pas d'import : chaque revue se prépare à l'écran à partir des données reprises.</v>
       </c>
     </row>
     <row r="25">
@@ -823,13 +823,13 @@
         <v>(saisie à l'écran)</v>
       </c>
       <c r="C25" t="str">
-        <v>Entreprises extérieures</v>
+        <v>Signalements</v>
       </c>
       <c r="D25" t="str">
-        <v>Entreprises extérieures</v>
+        <v>Signalements</v>
       </c>
       <c r="E25" t="str">
-        <v>Pas d'import : une fiche par intervention.</v>
+        <v>Pas d'import : chaque presque-accident se signale à l'écran ; un historique se reprend au Registre AT/MP (type « Presque accident »).</v>
       </c>
     </row>
     <row r="26">
@@ -840,13 +840,13 @@
         <v>(saisie à l'écran)</v>
       </c>
       <c r="C26" t="str">
-        <v>Base documentaire</v>
+        <v>Entreprises extérieures</v>
       </c>
       <c r="D26" t="str">
-        <v>Base documentaire</v>
+        <v>Entreprises extérieures</v>
       </c>
       <c r="E26" t="str">
-        <v>Pas d'import : fiches et documents se saisissent à l'écran.</v>
+        <v>Pas d'import : une fiche par intervention.</v>
       </c>
     </row>
     <row r="27">
@@ -857,13 +857,13 @@
         <v>(saisie à l'écran)</v>
       </c>
       <c r="C27" t="str">
-        <v>Stock et lavages des EPI</v>
+        <v>Base documentaire</v>
       </c>
       <c r="D27" t="str">
-        <v>EPI &amp; Dotation</v>
+        <v>Base documentaire</v>
       </c>
       <c r="E27" t="str">
-        <v>Pas d'import pour ces deux onglets.</v>
+        <v>Pas d'import : fiches et documents se saisissent à l'écran.</v>
       </c>
     </row>
     <row r="28">
@@ -874,18 +874,35 @@
         <v>(saisie à l'écran)</v>
       </c>
       <c r="C28" t="str">
+        <v>Stock et lavages des EPI</v>
+      </c>
+      <c r="D28" t="str">
+        <v>EPI &amp; Dotation</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Pas d'import pour ces deux onglets.</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>—</v>
+      </c>
+      <c r="B29" t="str">
+        <v>(saisie à l'écran)</v>
+      </c>
+      <c r="C29" t="str">
         <v>Rendez-vous médicaux</v>
       </c>
-      <c r="D28" t="str">
+      <c r="D29" t="str">
         <v>Santé &amp; Visites → Agenda</v>
       </c>
-      <c r="E28" t="str">
+      <c r="E29" t="str">
         <v>Pas d'import : l'agenda démarre à la mise en service.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E29"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>